<commit_message>
gee, forgot to add a bunch of files for the last commit, plus fixes to 2023 results (and exporting full float values)
</commit_message>
<xml_diff>
--- a/legacy/nola_2023_results.xlsx
+++ b/legacy/nola_2023_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="1-Seed Draw" sheetId="1" state="visible" r:id="rId3"/>
@@ -1085,7 +1085,7 @@
   <dimension ref="A1:B34"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.66"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1702,7 +1702,7 @@
   <dimension ref="A1:X36"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="10.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="6" width="7.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="8.37"/>
@@ -4639,7 +4639,7 @@
         <v>0.5</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.435</v>
+        <v>0.475</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4765,7 +4765,7 @@
         <v>0.375</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>0.44</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
complete legacy/validate script, verified with 2023 results
</commit_message>
<xml_diff>
--- a/legacy/nola_2023_results.xlsx
+++ b/legacy/nola_2023_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="1-Seed Draw" sheetId="1" state="visible" r:id="rId3"/>
@@ -15,7 +15,8 @@
     <sheet name="5-Team Pairings" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="6-Team Bracket" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="7-Team Scores" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="8-Team Results" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="8-Playoff Scores" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="9-Final Results" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="249">
   <si>
     <t xml:space="preserve">Num</t>
   </si>
@@ -653,16 +654,16 @@
     <t xml:space="preserve">4A,5B</t>
   </si>
   <si>
-    <t xml:space="preserve">5A,4B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6A,3B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7A,2B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8A,1B</t>
+    <t xml:space="preserve">4B,5A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3B,6A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2B,7A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1B,8A</t>
   </si>
   <si>
     <t xml:space="preserve">Team</t>
@@ -765,6 +766,15 @@
   </si>
   <si>
     <t xml:space="preserve">Final Rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FF Matches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FF Win Pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FF Pts Pct</t>
   </si>
 </sst>
 </file>
@@ -854,7 +864,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -896,6 +906,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7180,15 +7194,382 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:T5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="24.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="6" width="7.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="8.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="6" width="5.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="6" width="8.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="13" style="6" width="5.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="6" width="9.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="7" width="7.88"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <f aca="false">COUNTIF(F2:K2,10)</f>
+        <v>4</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <f aca="false">COUNTIF(M2:R2,10)</f>
+        <v>1</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <f aca="false">C2/(C2+D2)</f>
+        <v>0.8</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <f aca="false">SUM(F2:K2)</f>
+        <v>44</v>
+      </c>
+      <c r="M2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="P2" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q2" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="R2" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S2" s="6" t="n">
+        <f aca="false">SUM(M2:R2)</f>
+        <v>31</v>
+      </c>
+      <c r="T2" s="7" t="n">
+        <f aca="false">L2/(L2+S2)</f>
+        <v>0.586666666666667</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <f aca="false">COUNTIF(F3:K3,10)</f>
+        <v>3</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <f aca="false">COUNTIF(M3:R3,10)</f>
+        <v>3</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <f aca="false">C3/(C3+D3)</f>
+        <v>0.5</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <f aca="false">SUM(F3:K3)</f>
+        <v>45</v>
+      </c>
+      <c r="M3" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N3" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P3" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <f aca="false">SUM(M3:R3)</f>
+        <v>45</v>
+      </c>
+      <c r="T3" s="7" t="n">
+        <f aca="false">L3/(L3+S3)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <f aca="false">COUNTIF(F4:K4,10)</f>
+        <v>1</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <f aca="false">COUNTIF(M4:R4,10)</f>
+        <v>2</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <f aca="false">C4/(C4+D4)</f>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <f aca="false">SUM(F4:K4)</f>
+        <v>21</v>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="S4" s="6" t="n">
+        <f aca="false">SUM(M4:R4)</f>
+        <v>24</v>
+      </c>
+      <c r="T4" s="7" t="n">
+        <f aca="false">L4/(L4+S4)</f>
+        <v>0.466666666666667</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <f aca="false">COUNTIF(F5:K5,10)</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <f aca="false">COUNTIF(M5:R5,10)</f>
+        <v>2</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <f aca="false">C5/(C5+D5)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <f aca="false">SUM(F5:K5)</f>
+        <v>10</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <f aca="false">SUM(M5:R5)</f>
+        <v>20</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <f aca="false">L5/(L5+S5)</f>
+        <v>0.333333333333333</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="24.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10.75"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>245</v>
       </c>
@@ -7203,6 +7584,15 @@
       </c>
       <c r="E1" s="3" t="s">
         <v>130</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7217,6 +7607,9 @@
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
+      <c r="F2" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
@@ -7230,6 +7623,9 @@
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
+      <c r="F3" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
@@ -7243,6 +7639,15 @@
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
+      <c r="F4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>0.477</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
@@ -7256,6 +7661,15 @@
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
+      <c r="F5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">

</xml_diff>

<commit_message>
slight cleanup for tie-break logging, add annotations and minor fixups for 2023 and 2024 results
</commit_message>
<xml_diff>
--- a/legacy/nola_2023_results.xlsx
+++ b/legacy/nola_2023_results.xlsx
@@ -27,6 +27,158 @@
 </workbook>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="E4" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Note that this is mistakenly represented at 0.5 in the Seeding Round Results poster (see worksheet 4)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Changed to 6 from 2, based on other player scores</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Changed to 39 from 35, based on updated round 8 score</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N4" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Changed to 51 from 41 (math error)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Changed to 48 from 47 (math error)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Changed to 5 from 10, based on other player scores</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Changed to 46 from 51, based on corrected round 7 score</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X4" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Note that this is mistakenly represented at 0.466 in the Seeding Round Results poster (see worksheet 4)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Should really be position 9 based on Win Pct and Pts Pct (with current positions 9-17 all shifted down by 1)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Should be 0.571 (see worksheet 3)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Should be 0.520 (see worksheet 3)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="249">
   <si>
@@ -785,7 +937,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -820,6 +972,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -905,11 +1062,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1972,7 +2129,7 @@
         <f aca="false">COUNTIF(O4:V4,10)</f>
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="10" t="n">
         <f aca="false">C4/(C4+D4)</f>
         <v>0.571428571428571</v>
       </c>
@@ -2030,7 +2187,7 @@
       <c r="W4" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="X4" s="7" t="n">
+      <c r="X4" s="10" t="n">
         <f aca="false">N4/(N4+W4)</f>
         <v>0.520408163265306</v>
       </c>
@@ -4389,6 +4546,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4660,13 +4818,13 @@
       <c r="A19" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C19" s="10" t="n">
+      <c r="B19" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <v>0.466</v>
       </c>
     </row>
@@ -4888,6 +5046,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -7564,12 +7723,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="24.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="5" width="12.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="5" width="11.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="5" width="10.75"/>
   </cols>
   <sheetData>
-    <row r="1" s="11" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>245</v>
       </c>
@@ -7585,13 +7744,13 @@
       <c r="E1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="3" t="s">
         <v>248</v>
       </c>
     </row>
@@ -7607,7 +7766,7 @@
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7623,7 +7782,7 @@
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7639,13 +7798,13 @@
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.333</v>
       </c>
-      <c r="H4" s="0" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.477</v>
       </c>
     </row>
@@ -7661,13 +7820,13 @@
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="0" t="n">
+      <c r="H5" s="5" t="n">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
annotations and slight fixup for legacy 2023 and 2024 results
</commit_message>
<xml_diff>
--- a/legacy/nola_2023_results.xlsx
+++ b/legacy/nola_2023_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="1-Seed Draw" sheetId="1" state="visible" r:id="rId3"/>
@@ -2109,7 +2109,7 @@
       <c r="W3" s="6" t="n">
         <v>64</v>
       </c>
-      <c r="X3" s="7" t="n">
+      <c r="X3" s="10" t="n">
         <f aca="false">N3/(N3+W3)</f>
         <v>0.378640776699029</v>
       </c>
@@ -2265,7 +2265,7 @@
       <c r="W5" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="X5" s="7" t="n">
+      <c r="X5" s="10" t="n">
         <f aca="false">N5/(N5+W5)</f>
         <v>0.504</v>
       </c>
@@ -3279,7 +3279,7 @@
       <c r="W18" s="9" t="n">
         <v>46</v>
       </c>
-      <c r="X18" s="7" t="n">
+      <c r="X18" s="10" t="n">
         <f aca="false">N18/(N18+W18)</f>
         <v>0.610169491525424</v>
       </c>

</xml_diff>

<commit_message>
small formatting tweaks to legacy tournament data (for consistency)
</commit_message>
<xml_diff>
--- a/legacy/nola_2023_results.xlsx
+++ b/legacy/nola_2023_results.xlsx
@@ -2265,7 +2265,7 @@
       <c r="W5" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="X5" s="10" t="n">
+      <c r="X5" s="7" t="n">
         <f aca="false">N5/(N5+W5)</f>
         <v>0.504</v>
       </c>
@@ -2343,7 +2343,7 @@
       <c r="W6" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="X6" s="7" t="n">
+      <c r="X6" s="10" t="n">
         <f aca="false">N6/(N6+W6)</f>
         <v>0.424778761061947</v>
       </c>
@@ -4560,6 +4560,7 @@
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="17.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="9.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5059,9 +5060,13 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.25"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="18.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="5" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.77"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="4.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="5" width="24.77"/>
   </cols>
   <sheetData>
@@ -7357,7 +7362,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="24.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="4" width="15.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="6" width="7.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="8.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="6" width="5.46"/>
@@ -7723,9 +7728,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="4" width="24.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="5" width="12.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="5" width="11.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="5" width="10.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="10.33"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="5" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>